<commit_message>
standardize_dates modified, also has been added prints to show feedback of the process
</commit_message>
<xml_diff>
--- a/output/sales_report.xlsx
+++ b/output/sales_report.xlsx
@@ -854,10 +854,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1340</v>
+        <v>890</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">

</xml_diff>